<commit_message>
Update: decorated cavern & upper chambers
</commit_message>
<xml_diff>
--- a/Docs/Cells and References.xlsx
+++ b/Docs/Cells and References.xlsx
@@ -1,15 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etste\Documents\Projects\Mods\Morrowind\shrine-of-separation\Docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DD28666-C3F9-4A97-B86D-67F6A69A3496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Cells" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Containers" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="NPCs" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="Creatures" sheetId="4" r:id="rId7"/>
+    <sheet name="Cells" sheetId="1" r:id="rId1"/>
+    <sheet name="Containers" sheetId="2" r:id="rId2"/>
+    <sheet name="NPCs" sheetId="3" r:id="rId3"/>
+    <sheet name="Creatures" sheetId="4" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -163,32 +172,34 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -196,50 +207,56 @@
         <bgColor rgb="FFF4CCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor rgb="FFF4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -429,22 +446,25 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A2:Z6"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="18.88"/>
-    <col customWidth="1" min="3" max="3" width="31.38"/>
-    <col customWidth="1" min="6" max="6" width="25.13"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" customWidth="1"/>
+    <col min="6" max="6" width="25.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -461,15 +481,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="2"/>
@@ -495,8 +515,8 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4">
-      <c r="A4" s="2"/>
+    <row r="4" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
@@ -506,33 +526,33 @@
       <c r="D4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="2"/>
+      <c r="E4" s="3"/>
       <c r="F4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
-      <c r="W4" s="2"/>
-      <c r="X4" s="2"/>
-      <c r="Y4" s="2"/>
-      <c r="Z4" s="2"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+    </row>
+    <row r="5" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
       <c r="B5" s="3" t="s">
         <v>11</v>
       </c>
@@ -542,44 +562,44 @@
       <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="2"/>
+      <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
-      <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-      <c r="Y5" s="2"/>
-      <c r="Z5" s="2"/>
-    </row>
-    <row r="6">
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E6" s="2"/>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G6" s="2"/>
@@ -604,23 +624,24 @@
       <c r="Z6" s="2"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A2:Z7"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="18.88"/>
-    <col customWidth="1" min="3" max="3" width="31.38"/>
-    <col customWidth="1" min="4" max="5" width="18.88"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" customWidth="1"/>
+    <col min="4" max="5" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -634,18 +655,18 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="2"/>
@@ -670,18 +691,18 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F4" s="2"/>
@@ -706,18 +727,18 @@
       <c r="Y4" s="2"/>
       <c r="Z4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F5" s="2"/>
@@ -742,18 +763,18 @@
       <c r="Y5" s="2"/>
       <c r="Z5" s="2"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>29</v>
       </c>
       <c r="F6" s="2"/>
@@ -778,18 +799,18 @@
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F7" s="2"/>
@@ -815,22 +836,23 @@
       <c r="Z7" s="2"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A2:Z4"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="18.88"/>
-    <col customWidth="1" min="3" max="3" width="31.38"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -841,15 +863,15 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>36</v>
       </c>
       <c r="E3" s="2"/>
@@ -875,15 +897,15 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>36</v>
       </c>
       <c r="E4" s="2"/>
@@ -910,22 +932,23 @@
       <c r="Z4" s="2"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A2:Z5"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="18.88"/>
-    <col customWidth="1" min="3" max="3" width="31.38"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -936,15 +959,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>41</v>
       </c>
       <c r="E3" s="2"/>
@@ -970,15 +993,15 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>44</v>
       </c>
       <c r="E4" s="2"/>
@@ -1004,15 +1027,15 @@
       <c r="Y4" s="2"/>
       <c r="Z4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>47</v>
       </c>
       <c r="E5" s="2"/>
@@ -1039,6 +1062,6 @@
       <c r="Z5" s="2"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add: start of quest
</commit_message>
<xml_diff>
--- a/Docs/Cells and References.xlsx
+++ b/Docs/Cells and References.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etste\Documents\Projects\Mods\Morrowind\shrine-of-separation\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C29E183D-D56B-4A9C-B36B-0AC515F6935E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C982D8-6B7A-4E33-9555-F23D8DEB0407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cells" sheetId="1" r:id="rId1"/>
     <sheet name="Containers" sheetId="2" r:id="rId2"/>
-    <sheet name="NPCs" sheetId="3" r:id="rId3"/>
-    <sheet name="Creatures" sheetId="4" r:id="rId4"/>
+    <sheet name="Equipment" sheetId="5" r:id="rId3"/>
+    <sheet name="NPCs" sheetId="3" r:id="rId4"/>
+    <sheet name="Creatures" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="53">
   <si>
     <t>ID</t>
   </si>
@@ -173,13 +174,22 @@
   </si>
   <si>
     <t>Golden Saint</t>
+  </si>
+  <si>
+    <t>tlvsos_ring</t>
+  </si>
+  <si>
+    <t>Artoria's Ring of Rescue</t>
+  </si>
+  <si>
+    <t>Ring</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -197,6 +207,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -250,7 +268,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -258,6 +276,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -501,16 +520,434 @@
         <v>4</v>
       </c>
     </row>
+    <row r="3" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
+    </row>
+    <row r="4" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+    </row>
+    <row r="5" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
+    </row>
+    <row r="6" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
+      <c r="U6" s="3"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="3"/>
+      <c r="X6" s="3"/>
+      <c r="Y6" s="3"/>
+      <c r="Z6" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A2:Z7"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" customWidth="1"/>
+    <col min="4" max="5" width="18.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="2"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="2"/>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4439836A-187B-49EC-8F6E-7B66CF7EDF0A}">
+  <dimension ref="B2:D3"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="24.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A2:Z4"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -535,388 +972,6 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3"/>
-      <c r="Z4" s="3"/>
-    </row>
-    <row r="5" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="3"/>
-      <c r="Y5" s="3"/>
-      <c r="Z5" s="3"/>
-    </row>
-    <row r="6" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
-      <c r="X6" s="3"/>
-      <c r="Y6" s="3"/>
-      <c r="Z6" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A2:Z7"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="18.88671875" customWidth="1"/>
-    <col min="3" max="3" width="31.33203125" customWidth="1"/>
-    <col min="4" max="5" width="18.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
-      <c r="W4" s="2"/>
-      <c r="X4" s="2"/>
-      <c r="Y4" s="2"/>
-      <c r="Z4" s="2"/>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
-      <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-      <c r="Y5" s="2"/>
-      <c r="Z5" s="2"/>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
-      <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
-      <c r="W6" s="2"/>
-      <c r="X6" s="2"/>
-      <c r="Y6" s="2"/>
-      <c r="Z6" s="2"/>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="2"/>
-      <c r="W7" s="2"/>
-      <c r="X7" s="2"/>
-      <c r="Y7" s="2"/>
-      <c r="Z7" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A2:Z4"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="18.88671875" customWidth="1"/>
-    <col min="3" max="3" width="31.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
-    </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
@@ -956,7 +1011,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -968,7 +1023,7 @@
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -979,7 +1034,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" s="6" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
         <v>39</v>
@@ -1013,7 +1068,7 @@
       <c r="Y3" s="5"/>
       <c r="Z3" s="5"/>
     </row>
-    <row r="4" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" s="6" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="5" t="s">
         <v>42</v>
@@ -1047,7 +1102,7 @@
       <c r="Y4" s="5"/>
       <c r="Z4" s="5"/>
     </row>
-    <row r="5" spans="1:26" s="4" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" s="4" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3" t="s">
         <v>45</v>

</xml_diff>

<commit_message>
Update: Opening to dungeon, populate cavern
Add: Ebony Naginata
</commit_message>
<xml_diff>
--- a/Docs/Cells and References.xlsx
+++ b/Docs/Cells and References.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etste\Documents\Projects\Mods\Morrowind\shrine-of-separation\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C982D8-6B7A-4E33-9555-F23D8DEB0407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1FF448D-163E-4ACF-83E7-78B87F1B88AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
   <si>
     <t>ID</t>
   </si>
@@ -183,6 +183,12 @@
   </si>
   <si>
     <t>Ring</t>
+  </si>
+  <si>
+    <t>tlvsos_ringmartialprowess</t>
+  </si>
+  <si>
+    <t>Ring of Martial Prowess</t>
   </si>
 </sst>
 </file>
@@ -730,41 +736,41 @@
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
-      <c r="W4" s="2"/>
-      <c r="X4" s="2"/>
-      <c r="Y4" s="2"/>
-      <c r="Z4" s="2"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
@@ -881,10 +887,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4439836A-187B-49EC-8F6E-7B66CF7EDF0A}">
-  <dimension ref="B2:D3"/>
+  <dimension ref="B2:D4"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="2" max="2" width="23.109375" customWidth="1"/>
     <col min="3" max="3" width="24.77734375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -907,6 +913,17 @@
         <v>51</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>52</v>
       </c>
     </row>
@@ -972,39 +989,39 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
-      <c r="W4" s="2"/>
-      <c r="X4" s="2"/>
-      <c r="Y4" s="2"/>
-      <c r="Z4" s="2"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1034,39 +1051,39 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:26" s="6" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5" t="s">
+    <row r="3" spans="1:26" s="4" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
-      <c r="X3" s="5"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="5"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
     </row>
     <row r="4" spans="1:26" s="6" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>

</xml_diff>

<commit_message>
Update: populate chambers, scripted boss gates
</commit_message>
<xml_diff>
--- a/Docs/Cells and References.xlsx
+++ b/Docs/Cells and References.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etste\Documents\Projects\Mods\Morrowind\shrine-of-separation\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1FF448D-163E-4ACF-83E7-78B87F1B88AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5887CDAC-DC0C-414E-96A3-85F9D80F3F51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cells" sheetId="1" r:id="rId1"/>
@@ -224,7 +224,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -249,18 +249,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor rgb="FFF4CCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -274,14 +262,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -772,41 +758,41 @@
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
+    <row r="5" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
-      <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-      <c r="Y5" s="2"/>
-      <c r="Z5" s="2"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
@@ -895,13 +881,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="5" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1085,39 +1071,39 @@
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
     </row>
-    <row r="4" spans="1:26" s="6" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5" t="s">
+    <row r="4" spans="1:26" s="4" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
-      <c r="T4" s="5"/>
-      <c r="U4" s="5"/>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
-      <c r="X4" s="5"/>
-      <c r="Y4" s="5"/>
-      <c r="Z4" s="5"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
     </row>
     <row r="5" spans="1:26" s="4" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>

</xml_diff>